<commit_message>
docs(capstone): actualizar Gantt 2.3, UML 1.3 y guia 1.1
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Carta_Gantt_seb.acevedoa_mart.espinozam_je.fernandezm_Aprueba_ModuloPreguntas.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Carta_Gantt_seb.acevedoa_mart.espinozam_je.fernandezm_Aprueba_ModuloPreguntas.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="310">
   <si>
     <t>PLAN DE ITERACIONES - EXTREME PROGRAMMING</t>
   </si>
@@ -930,6 +930,27 @@
   </si>
   <si>
     <t>A = actualización del documento por cambios del proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semana 1: 10/08/2026 · Semana 18: 12/12/2026 · Diez iteraciones semanales agrupadas en tres entregas funcionales · Versión 2.3 · 18/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iteración 7 · Cuota diaria y desbloqueo, y correcciones de la aceptación de la iteración 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuota diaria escalonada y pantalla de desbloqueo, y correcciones de la aceptación de la iteración 6 (T-43 y T-56 a T-59)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cierre de la iteración 6 y de la entrega funcional 2: la habilidad evaluada (HU-06) se acepta el 18/10/2026 con la prueba T-48, con 5 de 5 puntos. La iteración 7 incorpora las correcciones de la aceptación (T-43 y T-56 a T-59), sin cambiar sus puntos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iteración 7 · Cuota diaria y desbloqueo, y correcciones de la iteración 6</t>
   </si>
 </sst>
 </file>
@@ -2086,7 +2107,7 @@
     </row>
     <row r="3">
       <c r="C3" s="4" t="s">
-        <v>37</v>
+        <v>303</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -3299,7 +3320,7 @@
         <v>242</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>243</v>
+        <v>304</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>25</v>
@@ -6765,7 +6786,7 @@
         <v>58</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>59</v>
+        <v>305</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>60</v>
@@ -8835,7 +8856,7 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="7" t="s">
-        <v>243</v>
+        <v>309</v>
       </c>
       <c r="B35" s="6">
         <f t="shared" si="1"/>
@@ -11649,6 +11670,17 @@
         <v>269</v>
       </c>
     </row>
+    <row r="8" ht="75.0" customHeight="1">
+      <c r="A8" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>

</xml_diff>